<commit_message>
Updating manual matches for EPA to EIA data (includes unit modification)
</commit_message>
<xml_diff>
--- a/manual_matches.xlsx
+++ b/manual_matches.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\capd_eia_crosswalk\users\gofortht\crosswalk_repo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\capd_eia_crosswalk\users\zhangm\camd-eia-crosswalk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C94E93B8-E055-4CA7-BC07-E057045814CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8704C065-C8D8-4645-959A-26DE4D9B67D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5460" yWindow="1170" windowWidth="28800" windowHeight="7800" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="unit_manual_matches" sheetId="1" r:id="rId1"/>
     <sheet name="unit_manual_excluded" sheetId="2" r:id="rId2"/>
     <sheet name="plant_id_manual_matches" sheetId="3" r:id="rId3"/>
-    <sheet name="further_research" sheetId="5" r:id="rId4"/>
-    <sheet name="Sheet Descriptions" sheetId="4" r:id="rId5"/>
+    <sheet name="plant_id_epa_to_eia" sheetId="6" r:id="rId4"/>
+    <sheet name="further_research" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet Descriptions" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">plant_id_manual_matches!$A$1:$D$1</definedName>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="513">
   <si>
     <t>EIA_PLANT_ID</t>
   </si>
@@ -1531,6 +1532,54 @@
   </si>
   <si>
     <t>UNIT2</t>
+  </si>
+  <si>
+    <t>epa_plant_name</t>
+  </si>
+  <si>
+    <t>epa_plant_id</t>
+  </si>
+  <si>
+    <t>epa_unit_id</t>
+  </si>
+  <si>
+    <t>eia_plant_name</t>
+  </si>
+  <si>
+    <t>eia_plant_id</t>
+  </si>
+  <si>
+    <t>eia_unit_id</t>
+  </si>
+  <si>
+    <t>AES Puerto Rico, LP</t>
+  </si>
+  <si>
+    <t>AES Puerto Rico</t>
+  </si>
+  <si>
+    <t>Aguirre Steam Power Plant</t>
+  </si>
+  <si>
+    <t>Aguirre Plant</t>
+  </si>
+  <si>
+    <t>Costa Sur Steam Power Plant</t>
+  </si>
+  <si>
+    <t>Costa Sur Plant</t>
+  </si>
+  <si>
+    <t>San Juan Steam Power Plant</t>
+  </si>
+  <si>
+    <t>Central San Juan Plant</t>
+  </si>
+  <si>
+    <t>Palo Seco Steam Power Plant</t>
+  </si>
+  <si>
+    <t>Palo Seco Plant</t>
   </si>
 </sst>
 </file>
@@ -9364,6 +9413,356 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02294E30-E5CA-4696-82B9-6506C2DB56DE}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>497</v>
+      </c>
+      <c r="B1" t="s">
+        <v>498</v>
+      </c>
+      <c r="C1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1" t="s">
+        <v>500</v>
+      </c>
+      <c r="E1" t="s">
+        <v>501</v>
+      </c>
+      <c r="F1" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>503</v>
+      </c>
+      <c r="B2">
+        <v>880102</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>504</v>
+      </c>
+      <c r="E2">
+        <v>61082</v>
+      </c>
+      <c r="F2" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B3">
+        <v>880102</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>504</v>
+      </c>
+      <c r="E3">
+        <v>61082</v>
+      </c>
+      <c r="F3" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>505</v>
+      </c>
+      <c r="B4">
+        <v>880105</v>
+      </c>
+      <c r="C4" t="s">
+        <v>481</v>
+      </c>
+      <c r="D4" t="s">
+        <v>506</v>
+      </c>
+      <c r="E4">
+        <v>61146</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>505</v>
+      </c>
+      <c r="B5">
+        <v>880105</v>
+      </c>
+      <c r="C5" t="s">
+        <v>482</v>
+      </c>
+      <c r="D5" t="s">
+        <v>506</v>
+      </c>
+      <c r="E5">
+        <v>61146</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>507</v>
+      </c>
+      <c r="B6">
+        <v>880104</v>
+      </c>
+      <c r="C6" t="s">
+        <v>483</v>
+      </c>
+      <c r="D6" t="s">
+        <v>508</v>
+      </c>
+      <c r="E6">
+        <v>61147</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>507</v>
+      </c>
+      <c r="B7">
+        <v>880104</v>
+      </c>
+      <c r="C7" t="s">
+        <v>484</v>
+      </c>
+      <c r="D7" t="s">
+        <v>508</v>
+      </c>
+      <c r="E7">
+        <v>61147</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>507</v>
+      </c>
+      <c r="B8">
+        <v>880104</v>
+      </c>
+      <c r="C8" t="s">
+        <v>485</v>
+      </c>
+      <c r="D8" t="s">
+        <v>508</v>
+      </c>
+      <c r="E8">
+        <v>61147</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>507</v>
+      </c>
+      <c r="B9">
+        <v>880104</v>
+      </c>
+      <c r="C9" t="s">
+        <v>486</v>
+      </c>
+      <c r="D9" t="s">
+        <v>508</v>
+      </c>
+      <c r="E9">
+        <v>61147</v>
+      </c>
+      <c r="F9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>509</v>
+      </c>
+      <c r="B10">
+        <v>880106</v>
+      </c>
+      <c r="C10" t="s">
+        <v>487</v>
+      </c>
+      <c r="D10" t="s">
+        <v>510</v>
+      </c>
+      <c r="E10">
+        <v>61148</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>509</v>
+      </c>
+      <c r="B11">
+        <v>880106</v>
+      </c>
+      <c r="C11" t="s">
+        <v>488</v>
+      </c>
+      <c r="D11" t="s">
+        <v>510</v>
+      </c>
+      <c r="E11">
+        <v>61148</v>
+      </c>
+      <c r="F11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>509</v>
+      </c>
+      <c r="B12">
+        <v>880107</v>
+      </c>
+      <c r="C12" t="s">
+        <v>489</v>
+      </c>
+      <c r="D12" t="s">
+        <v>510</v>
+      </c>
+      <c r="E12">
+        <v>61148</v>
+      </c>
+      <c r="F12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>509</v>
+      </c>
+      <c r="B13">
+        <v>880108</v>
+      </c>
+      <c r="C13" t="s">
+        <v>490</v>
+      </c>
+      <c r="D13" t="s">
+        <v>510</v>
+      </c>
+      <c r="E13">
+        <v>61148</v>
+      </c>
+      <c r="F13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>511</v>
+      </c>
+      <c r="B14">
+        <v>880103</v>
+      </c>
+      <c r="C14" t="s">
+        <v>491</v>
+      </c>
+      <c r="D14" t="s">
+        <v>512</v>
+      </c>
+      <c r="E14">
+        <v>61149</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>511</v>
+      </c>
+      <c r="B15">
+        <v>880103</v>
+      </c>
+      <c r="C15" t="s">
+        <v>492</v>
+      </c>
+      <c r="D15" t="s">
+        <v>512</v>
+      </c>
+      <c r="E15">
+        <v>61149</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>511</v>
+      </c>
+      <c r="B16">
+        <v>880103</v>
+      </c>
+      <c r="C16" t="s">
+        <v>493</v>
+      </c>
+      <c r="D16" t="s">
+        <v>512</v>
+      </c>
+      <c r="E16">
+        <v>61149</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>511</v>
+      </c>
+      <c r="B17">
+        <v>880103</v>
+      </c>
+      <c r="C17" t="s">
+        <v>494</v>
+      </c>
+      <c r="D17" t="s">
+        <v>512</v>
+      </c>
+      <c r="E17">
+        <v>61149</v>
+      </c>
+      <c r="F17">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EB1A3B7-CB0E-4C70-B712-DAB54E286D7C}">
   <dimension ref="A1:G112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10299,7 +10698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD10B953-F711-4F6E-8A1B-58F0D1356472}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10355,59 +10754,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2021-06-22T20:59:33+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF32AD688505FB45A4B74E8374DD655E" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="820e166eda12a2b21727580e35d4b1c4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="03c14dc6-992a-47d3-9648-df74221fc344" xmlns:ns6="434a65cb-19a2-4f64-81f9-c4c3497f5b4c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="73bb20789afc0d8257071bd90159119b" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -10844,44 +11190,60 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7F48335-9609-4D38-B63B-9A6620FE759C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="434a65cb-19a2-4f64-81f9-c4c3497f5b4c"/>
-    <ds:schemaRef ds:uri="03c14dc6-992a-47d3-9648-df74221fc344"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72D1F9EA-526B-4162-847E-36B5EC9F2951}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B99ED44-03A6-4635-B387-C99415CE560D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2021-06-22T20:59:33+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58D1E071-1F27-41E0-9A83-EBB1CE4676B1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10902,4 +11264,41 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B99ED44-03A6-4635-B387-C99415CE560D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72D1F9EA-526B-4162-847E-36B5EC9F2951}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7F48335-9609-4D38-B63B-9A6620FE759C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="434a65cb-19a2-4f64-81f9-c4c3497f5b4c"/>
+    <ds:schemaRef ds:uri="03c14dc6-992a-47d3-9648-df74221fc344"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>